<commit_message>
Updated BOM with Honeywell PB
</commit_message>
<xml_diff>
--- a/3xCarbide Permit ILK(BOM).xlsx
+++ b/3xCarbide Permit ILK(BOM).xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jinop\Documents\_KiCADwork\GitWork\KiCAD_3xCarbide-ILK\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{6CE25C13-DA78-4DC1-ACF5-8D2E98AC0373}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{B94FE166-8543-46E9-A163-F419CE67A60C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11265" yWindow="-18960" windowWidth="27345" windowHeight="14115" xr2:uid="{342D2514-BD5C-4A37-9260-FFF5CCCA79E4}"/>
+    <workbookView xWindow="11265" yWindow="-18960" windowWidth="27345" windowHeight="14115" xr2:uid="{76CD675D-07B2-4316-8CD2-77D8AF8CA5C1}"/>
   </bookViews>
   <sheets>
     <sheet name="3xCarbide Permit ILK" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="73">
   <si>
     <t>Reference</t>
   </si>
@@ -46,6 +46,21 @@
     <t>Datasheet</t>
   </si>
   <si>
+    <t>LED1,LED2,LED3,LED4,LED5,LED6</t>
+  </si>
+  <si>
+    <t>GRN/24V</t>
+  </si>
+  <si>
+    <t>TT Electronics</t>
+  </si>
+  <si>
+    <t>LED GREEN CLEAR 5MM T/H</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/tt-electronics-optek-technology/OVLFG3C7/827117</t>
+  </si>
+  <si>
     <t>TB-A3,TB-A4,TB-B3,TB-B4,TB3,TB4</t>
   </si>
   <si>
@@ -70,13 +85,16 @@
     <t>SW1,SW2,SW3,SW4,SW5,SW6</t>
   </si>
   <si>
-    <t>18535CD</t>
-  </si>
-  <si>
-    <t>APEM Inc.</t>
-  </si>
-  <si>
-    <t>SWITCH PUSH SPDT 0.1A 30V, Electrical Life 60,000 Cycles, 100 mA(DC)</t>
+    <t>2PB11</t>
+  </si>
+  <si>
+    <t>Honeywell Sensing</t>
+  </si>
+  <si>
+    <t>PB Switch SPDT x 2 Standard Panel Mount, Rear</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/honeywell-sensing-and-productivity-solutions/2PB11/1248816</t>
   </si>
   <si>
     <t>SSR-StsA1,SSR-StsA2,SSR-StsA3</t>
@@ -124,21 +142,6 @@
     <t>https://www.mouser.com/datasheet/3/507/8/phoenix_contact_1523018_en.pdf</t>
   </si>
   <si>
-    <t>LED1,LED2,LED3,LED4,LED5,LED6</t>
-  </si>
-  <si>
-    <t>GRN/24V</t>
-  </si>
-  <si>
-    <t>TT Electronics</t>
-  </si>
-  <si>
-    <t>LED GREEN CLEAR 5MM T/H</t>
-  </si>
-  <si>
-    <t>https://www.digikey.com/en/products/detail/tt-electronics-optek-technology/OVLFG3C7/827117</t>
-  </si>
-  <si>
     <t>J7</t>
   </si>
   <si>
@@ -214,6 +217,15 @@
     <t>CONN TERM BLK DISCONN 10-30AWG Fuse Type: 6.3mm x 32mm</t>
   </si>
   <si>
+    <t>EDP1</t>
+  </si>
+  <si>
+    <t>Connector End Plate For CLIPLINE PT Series</t>
+  </si>
+  <si>
+    <t>https://www.phoenixcontact.com/en-us/products/end-cover-d-pt-15s-quattro-3208375?type=pdf</t>
+  </si>
+  <si>
     <t>DPM1,DPM2,DPM3</t>
   </si>
   <si>
@@ -227,12 +239,6 @@
   </si>
   <si>
     <t>https://www.automationdirect.com/adc/shopping/catalog/process_control_-a-_measurement/digital_panel_meters/analog_input/dpm1-a-2r-l</t>
-  </si>
-  <si>
-    <t>Sub</t>
-  </si>
-  <si>
-    <t>SUB</t>
   </si>
 </sst>
 </file>
@@ -720,13 +726,10 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="6" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1101,23 +1104,21 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1A4519C3-377B-448B-A9F0-854C754AC036}">
-  <dimension ref="A1:I17"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{784B577F-C214-4A25-AC07-E369FCA46145}">
+  <dimension ref="A1:H16"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="52.109375" customWidth="1"/>
-    <col min="2" max="2" width="13.88671875" style="3" customWidth="1"/>
-    <col min="5" max="5" width="14.88671875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="9.6640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="79.33203125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="126.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.88671875" customWidth="1"/>
+    <col min="3" max="3" width="13.44140625" customWidth="1"/>
+    <col min="5" max="5" width="17.109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="79.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
       <c r="C1" t="s">
@@ -1133,403 +1134,361 @@
         <v>5</v>
       </c>
       <c r="G1" t="s">
-        <v>69</v>
+        <v>6</v>
       </c>
       <c r="H1" t="s">
-        <v>6</v>
-      </c>
-      <c r="I1" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>8</v>
       </c>
-      <c r="B2" s="3">
+      <c r="B2">
         <v>6</v>
       </c>
       <c r="C2" t="s">
         <v>9</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>10</v>
       </c>
-      <c r="E2" t="s">
+      <c r="F2" s="1">
+        <v>0.44</v>
+      </c>
+      <c r="G2" t="s">
         <v>11</v>
       </c>
-      <c r="F2" s="1">
-        <v>1.83</v>
-      </c>
-      <c r="G2" s="1">
-        <f>B2*F2</f>
-        <v>10.98</v>
-      </c>
-      <c r="I2" t="s">
+      <c r="H2" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>13</v>
       </c>
-      <c r="B3" s="3">
+      <c r="B3">
         <v>6</v>
       </c>
       <c r="C3" t="s">
         <v>14</v>
       </c>
       <c r="D3" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="E3" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="F3" s="1">
         <v>1.83</v>
       </c>
-      <c r="G3" s="1">
-        <f t="shared" ref="G3:G15" si="0">B3*F3</f>
-        <v>10.98</v>
-      </c>
-      <c r="I3" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="H3" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B4">
+        <v>6</v>
+      </c>
+      <c r="C4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D4" t="s">
         <v>15</v>
       </c>
-      <c r="B4" s="3">
+      <c r="E4" t="s">
+        <v>16</v>
+      </c>
+      <c r="F4" s="1">
+        <v>1.83</v>
+      </c>
+      <c r="H4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>20</v>
+      </c>
+      <c r="B5">
         <v>6</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C5" t="s">
+        <v>21</v>
+      </c>
+      <c r="E5" t="s">
+        <v>22</v>
+      </c>
+      <c r="F5" s="1">
+        <v>165.16</v>
+      </c>
+      <c r="G5" t="s">
+        <v>23</v>
+      </c>
+      <c r="H5" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>25</v>
+      </c>
+      <c r="B6">
+        <v>3</v>
+      </c>
+      <c r="C6">
+        <v>2905293</v>
+      </c>
+      <c r="E6" t="s">
         <v>16</v>
       </c>
-      <c r="E4" t="s">
-        <v>17</v>
-      </c>
-      <c r="F4" s="1">
-        <v>12.96</v>
-      </c>
-      <c r="G4" s="1">
-        <f t="shared" si="0"/>
-        <v>77.760000000000005</v>
-      </c>
-      <c r="H4" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>19</v>
-      </c>
-      <c r="B5" s="3">
-        <v>3</v>
-      </c>
-      <c r="C5">
-        <v>2905293</v>
-      </c>
-      <c r="E5" t="s">
-        <v>11</v>
-      </c>
-      <c r="F5" s="1">
+      <c r="F6" s="1">
         <v>26.47</v>
       </c>
-      <c r="G5" s="1">
-        <f t="shared" si="0"/>
-        <v>79.41</v>
-      </c>
-      <c r="H5" t="s">
-        <v>20</v>
-      </c>
-      <c r="I5" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>22</v>
-      </c>
-      <c r="B6" s="3">
+      <c r="G6" t="s">
+        <v>26</v>
+      </c>
+      <c r="H6" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>28</v>
+      </c>
+      <c r="B7">
         <v>8</v>
       </c>
-      <c r="C6">
+      <c r="C7">
         <v>52511</v>
       </c>
-      <c r="E6" t="s">
-        <v>23</v>
-      </c>
-      <c r="F6" s="2">
+      <c r="E7" t="s">
+        <v>29</v>
+      </c>
+      <c r="F7" s="2">
         <v>63</v>
       </c>
-      <c r="G6" s="1">
-        <f t="shared" si="0"/>
-        <v>504</v>
-      </c>
-      <c r="H6" t="s">
-        <v>24</v>
-      </c>
-      <c r="I6" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>26</v>
-      </c>
-      <c r="B7" s="3">
+      <c r="G7" t="s">
+        <v>30</v>
+      </c>
+      <c r="H7" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>32</v>
+      </c>
+      <c r="B8">
         <v>5</v>
       </c>
-      <c r="C7">
+      <c r="C8">
         <v>3213014</v>
       </c>
-      <c r="E7" t="s">
-        <v>11</v>
-      </c>
-      <c r="F7" s="1">
+      <c r="E8" t="s">
+        <v>16</v>
+      </c>
+      <c r="F8" s="1">
         <v>0.69</v>
       </c>
-      <c r="G7" s="1">
-        <f t="shared" si="0"/>
-        <v>3.4499999999999997</v>
-      </c>
-      <c r="H7" t="s">
-        <v>27</v>
-      </c>
-      <c r="I7" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>29</v>
-      </c>
-      <c r="B8" s="3">
+      <c r="G8" t="s">
+        <v>33</v>
+      </c>
+      <c r="H8" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>35</v>
+      </c>
+      <c r="B9">
         <v>1</v>
       </c>
-      <c r="C8">
+      <c r="C9">
         <v>1523018</v>
       </c>
-      <c r="D8" t="s">
-        <v>30</v>
-      </c>
-      <c r="E8" t="s">
-        <v>31</v>
-      </c>
-      <c r="F8" s="1">
+      <c r="D9" t="s">
+        <v>36</v>
+      </c>
+      <c r="E9" t="s">
+        <v>37</v>
+      </c>
+      <c r="F9" s="1">
         <v>138.29</v>
       </c>
-      <c r="G8" s="1">
-        <f t="shared" si="0"/>
-        <v>138.29</v>
-      </c>
-      <c r="H8" t="s">
-        <v>32</v>
-      </c>
-      <c r="I8" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
-        <v>34</v>
-      </c>
-      <c r="B9" s="3">
-        <v>6</v>
-      </c>
-      <c r="C9" t="s">
-        <v>35</v>
-      </c>
-      <c r="E9" t="s">
-        <v>36</v>
-      </c>
-      <c r="F9" s="1">
-        <v>0.44</v>
-      </c>
-      <c r="G9" s="1">
-        <f t="shared" si="0"/>
-        <v>2.64</v>
+      <c r="G9" t="s">
+        <v>38</v>
       </c>
       <c r="H9" t="s">
-        <v>37</v>
-      </c>
-      <c r="I9" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>39</v>
-      </c>
-      <c r="B10" s="3">
+        <v>40</v>
+      </c>
+      <c r="B10">
         <v>1</v>
       </c>
       <c r="C10" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="E10" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="F10" s="1">
         <v>15.18</v>
       </c>
-      <c r="G10" s="1">
-        <f t="shared" si="0"/>
-        <v>15.18</v>
+      <c r="G10" t="s">
+        <v>43</v>
       </c>
       <c r="H10" t="s">
-        <v>42</v>
-      </c>
-      <c r="I10" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>44</v>
-      </c>
-      <c r="B11" s="3">
+        <v>45</v>
+      </c>
+      <c r="B11">
         <v>4</v>
       </c>
       <c r="C11" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="E11" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="F11" s="1">
         <v>24.98</v>
       </c>
-      <c r="G11" s="1">
-        <f t="shared" si="0"/>
-        <v>99.92</v>
+      <c r="G11" t="s">
+        <v>48</v>
       </c>
       <c r="H11" t="s">
-        <v>47</v>
-      </c>
-      <c r="I11" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>49</v>
-      </c>
-      <c r="B12" s="3">
+        <v>50</v>
+      </c>
+      <c r="B12">
         <v>2</v>
       </c>
       <c r="C12" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E12" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="F12" s="1">
         <v>22.73</v>
       </c>
-      <c r="G12" s="1">
-        <f t="shared" si="0"/>
-        <v>45.46</v>
+      <c r="G12" t="s">
+        <v>53</v>
       </c>
       <c r="H12" t="s">
-        <v>52</v>
-      </c>
-      <c r="I12" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>54</v>
-      </c>
-      <c r="B13" s="3">
+        <v>55</v>
+      </c>
+      <c r="B13">
         <v>1</v>
       </c>
       <c r="C13" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D13" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E13" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="F13" s="1">
         <v>6.16</v>
       </c>
-      <c r="G13" s="1">
-        <f t="shared" si="0"/>
-        <v>6.16</v>
+      <c r="G13" t="s">
+        <v>59</v>
       </c>
       <c r="H13" t="s">
-        <v>58</v>
-      </c>
-      <c r="I13" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>60</v>
-      </c>
-      <c r="B14" s="3">
+        <v>61</v>
+      </c>
+      <c r="B14">
         <v>2</v>
       </c>
       <c r="C14">
         <v>1880410000</v>
       </c>
       <c r="D14" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="E14" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="F14" s="1">
         <v>33.68</v>
       </c>
-      <c r="G14" s="1">
-        <f t="shared" si="0"/>
-        <v>67.36</v>
-      </c>
-      <c r="H14" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="G14" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>64</v>
-      </c>
-      <c r="B15" s="3">
-        <v>3</v>
-      </c>
-      <c r="C15" t="s">
         <v>65</v>
       </c>
+      <c r="B15">
+        <v>1</v>
+      </c>
+      <c r="C15">
+        <v>3208375</v>
+      </c>
       <c r="E15" t="s">
+        <v>16</v>
+      </c>
+      <c r="F15" s="1">
+        <v>0.84</v>
+      </c>
+      <c r="G15" t="s">
         <v>66</v>
-      </c>
-      <c r="F15" s="2">
-        <v>151</v>
-      </c>
-      <c r="G15" s="1">
-        <f t="shared" si="0"/>
-        <v>453</v>
       </c>
       <c r="H15" t="s">
         <v>67</v>
       </c>
-      <c r="I15" t="s">
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A17" t="s">
+      <c r="B16">
+        <v>3</v>
+      </c>
+      <c r="C16" t="s">
+        <v>69</v>
+      </c>
+      <c r="E16" t="s">
         <v>70</v>
       </c>
-      <c r="G17" s="1">
-        <f>SUM(G2:G15)</f>
-        <v>1514.59</v>
+      <c r="F16" s="2">
+        <v>151</v>
+      </c>
+      <c r="G16" t="s">
+        <v>71</v>
+      </c>
+      <c r="H16" t="s">
+        <v>72</v>
       </c>
     </row>
   </sheetData>

</xml_diff>